<commit_message>
chore: upload + test_fix
</commit_message>
<xml_diff>
--- a/LME/parser/lme/data/LME_db_new.xlsx
+++ b/LME/parser/lme/data/LME_db_new.xlsx
@@ -396,7 +396,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G1203"/>
+  <dimension ref="A1:G1202"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -26276,1172 +26276,1172 @@
     </row>
     <row r="1126" spans="1:7">
       <c r="A1126" s="2">
-        <v>46186</v>
+        <v>46188</v>
       </c>
       <c r="B1126">
-        <v>3536</v>
+        <v>3419.5</v>
       </c>
       <c r="C1126">
-        <v>13603</v>
+        <v>13714</v>
       </c>
       <c r="D1126">
-        <v>1957</v>
+        <v>1964</v>
       </c>
       <c r="E1126">
-        <v>17630</v>
+        <v>17810</v>
       </c>
       <c r="F1126">
-        <v>3557</v>
+        <v>3562</v>
       </c>
       <c r="G1126">
-        <v>53350</v>
+        <v>54650</v>
       </c>
     </row>
     <row r="1127" spans="1:7">
       <c r="A1127" s="2">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B1127">
-        <v>3419.5</v>
+        <v>3359</v>
       </c>
       <c r="C1127">
-        <v>13714</v>
+        <v>13682</v>
       </c>
       <c r="D1127">
-        <v>1964</v>
+        <v>1956</v>
       </c>
       <c r="E1127">
-        <v>17810</v>
+        <v>17630</v>
       </c>
       <c r="F1127">
-        <v>3562</v>
+        <v>3550</v>
       </c>
       <c r="G1127">
-        <v>54650</v>
+        <v>55150</v>
       </c>
     </row>
     <row r="1128" spans="1:7">
       <c r="A1128" s="2">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B1128">
-        <v>3359</v>
+        <v>3405.5</v>
       </c>
       <c r="C1128">
-        <v>13682</v>
+        <v>13736</v>
       </c>
       <c r="D1128">
-        <v>1956</v>
+        <v>1945</v>
       </c>
       <c r="E1128">
-        <v>17630</v>
+        <v>17820</v>
       </c>
       <c r="F1128">
-        <v>3550</v>
+        <v>3592</v>
       </c>
       <c r="G1128">
-        <v>55150</v>
+        <v>55400</v>
       </c>
     </row>
     <row r="1129" spans="1:7">
       <c r="A1129" s="2">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B1129">
-        <v>3405.5</v>
+        <v>3402</v>
       </c>
       <c r="C1129">
-        <v>13736</v>
+        <v>13612</v>
       </c>
       <c r="D1129">
         <v>1945</v>
       </c>
       <c r="E1129">
-        <v>17820</v>
+        <v>17770</v>
       </c>
       <c r="F1129">
-        <v>3592</v>
+        <v>3565</v>
       </c>
       <c r="G1129">
-        <v>55400</v>
+        <v>53455</v>
       </c>
     </row>
     <row r="1130" spans="1:7">
       <c r="A1130" s="2">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B1130">
-        <v>3402</v>
+        <v>3400</v>
       </c>
       <c r="C1130">
-        <v>13612</v>
+        <v>13530.5</v>
       </c>
       <c r="D1130">
-        <v>1945</v>
+        <v>1935</v>
       </c>
       <c r="E1130">
-        <v>17770</v>
+        <v>17590</v>
       </c>
       <c r="F1130">
-        <v>3565</v>
+        <v>3584.5</v>
       </c>
       <c r="G1130">
-        <v>53455</v>
+        <v>53200</v>
       </c>
     </row>
     <row r="1131" spans="1:7">
       <c r="A1131" s="2">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B1131">
-        <v>3400</v>
+        <v>3405</v>
       </c>
       <c r="C1131">
-        <v>13530.5</v>
+        <v>13642</v>
       </c>
       <c r="D1131">
-        <v>1935</v>
+        <v>1928.5</v>
       </c>
       <c r="E1131">
-        <v>17590</v>
+        <v>17640</v>
       </c>
       <c r="F1131">
-        <v>3584.5</v>
+        <v>3612.5</v>
       </c>
       <c r="G1131">
-        <v>53200</v>
+        <v>54995</v>
       </c>
     </row>
     <row r="1132" spans="1:7">
       <c r="A1132" s="2">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="B1132">
-        <v>3405</v>
+        <v>3263.5</v>
       </c>
       <c r="C1132">
-        <v>13642</v>
+        <v>13334</v>
       </c>
       <c r="D1132">
-        <v>1928.5</v>
+        <v>1910</v>
       </c>
       <c r="E1132">
-        <v>17640</v>
+        <v>17105</v>
       </c>
       <c r="F1132">
-        <v>3612.5</v>
+        <v>3503</v>
       </c>
       <c r="G1132">
-        <v>54995</v>
+        <v>51900</v>
       </c>
     </row>
     <row r="1133" spans="1:7">
       <c r="A1133" s="2">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="B1133">
-        <v>3263.5</v>
+        <v>3150</v>
       </c>
       <c r="C1133">
-        <v>13334</v>
+        <v>13181.5</v>
       </c>
       <c r="D1133">
-        <v>1910</v>
+        <v>1896</v>
       </c>
       <c r="E1133">
-        <v>17105</v>
+        <v>16610</v>
       </c>
       <c r="F1133">
-        <v>3503</v>
+        <v>3437</v>
       </c>
       <c r="G1133">
-        <v>51900</v>
+        <v>49550</v>
       </c>
     </row>
     <row r="1134" spans="1:7">
       <c r="A1134" s="2">
-        <v>46197</v>
+        <v>46198</v>
       </c>
       <c r="B1134">
-        <v>3150</v>
+        <v>3132</v>
       </c>
       <c r="C1134">
-        <v>13181.5</v>
+        <v>13194</v>
       </c>
       <c r="D1134">
-        <v>1896</v>
+        <v>1894</v>
       </c>
       <c r="E1134">
-        <v>16610</v>
+        <v>16660</v>
       </c>
       <c r="F1134">
-        <v>3437</v>
+        <v>3432</v>
       </c>
       <c r="G1134">
-        <v>49550</v>
+        <v>50100</v>
       </c>
     </row>
     <row r="1135" spans="1:7">
       <c r="A1135" s="2">
-        <v>46198</v>
+        <v>46199</v>
       </c>
       <c r="B1135">
-        <v>3132</v>
+        <v>3164</v>
       </c>
       <c r="C1135">
-        <v>13194</v>
+        <v>13287</v>
       </c>
       <c r="D1135">
-        <v>1894</v>
+        <v>1880</v>
       </c>
       <c r="E1135">
-        <v>16660</v>
+        <v>16570</v>
       </c>
       <c r="F1135">
-        <v>3432</v>
+        <v>3460</v>
       </c>
       <c r="G1135">
-        <v>50100</v>
+        <v>50325</v>
       </c>
     </row>
     <row r="1136" spans="1:7">
       <c r="A1136" s="2">
-        <v>46199</v>
+        <v>46202</v>
       </c>
       <c r="B1136">
-        <v>3164</v>
+        <v>3160.5</v>
       </c>
       <c r="C1136">
-        <v>13287</v>
+        <v>13302.5</v>
       </c>
       <c r="D1136">
-        <v>1880</v>
+        <v>1871.5</v>
       </c>
       <c r="E1136">
-        <v>16570</v>
+        <v>16455</v>
       </c>
       <c r="F1136">
-        <v>3460</v>
+        <v>3491</v>
       </c>
       <c r="G1136">
-        <v>50325</v>
+        <v>51000</v>
       </c>
     </row>
     <row r="1137" spans="1:7">
       <c r="A1137" s="2">
-        <v>46202</v>
+        <v>46203</v>
       </c>
       <c r="B1137">
-        <v>3160.5</v>
+        <v>3105.5</v>
       </c>
       <c r="C1137">
-        <v>13302.5</v>
+        <v>13341</v>
       </c>
       <c r="D1137">
-        <v>1871.5</v>
+        <v>1845</v>
       </c>
       <c r="E1137">
-        <v>16455</v>
+        <v>16275</v>
       </c>
       <c r="F1137">
-        <v>3491</v>
+        <v>3565.5</v>
       </c>
       <c r="G1137">
-        <v>51000</v>
+        <v>51100</v>
       </c>
     </row>
     <row r="1138" spans="1:7">
       <c r="A1138" s="2">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B1138">
-        <v>3105.5</v>
+        <v>3075</v>
       </c>
       <c r="C1138">
-        <v>13341</v>
+        <v>13170</v>
       </c>
       <c r="D1138">
-        <v>1845</v>
+        <v>1840</v>
       </c>
       <c r="E1138">
-        <v>16275</v>
+        <v>16175</v>
       </c>
       <c r="F1138">
-        <v>3565.5</v>
+        <v>3529</v>
       </c>
       <c r="G1138">
-        <v>51100</v>
+        <v>51150</v>
       </c>
     </row>
     <row r="1139" spans="1:7">
       <c r="A1139" s="2">
-        <v>46204</v>
+        <v>46205</v>
       </c>
       <c r="B1139">
-        <v>3075</v>
+        <v>3061.5</v>
       </c>
       <c r="C1139">
-        <v>13170</v>
+        <v>13202</v>
       </c>
       <c r="D1139">
-        <v>1840</v>
+        <v>1828.5</v>
       </c>
       <c r="E1139">
-        <v>16175</v>
+        <v>16070</v>
       </c>
       <c r="F1139">
-        <v>3529</v>
+        <v>3475</v>
       </c>
       <c r="G1139">
-        <v>51150</v>
+        <v>51200</v>
       </c>
     </row>
     <row r="1140" spans="1:7">
       <c r="A1140" s="2">
-        <v>46205</v>
+        <v>46206</v>
       </c>
       <c r="B1140">
-        <v>3061.5</v>
+        <v>3080</v>
       </c>
       <c r="C1140">
-        <v>13202</v>
+        <v>13298.5</v>
       </c>
       <c r="D1140">
-        <v>1828.5</v>
+        <v>1851</v>
       </c>
       <c r="E1140">
-        <v>16070</v>
+        <v>16115</v>
       </c>
       <c r="F1140">
-        <v>3475</v>
+        <v>3546</v>
       </c>
       <c r="G1140">
-        <v>51200</v>
+        <v>52000</v>
       </c>
     </row>
     <row r="1141" spans="1:7">
       <c r="A1141" s="2">
-        <v>46206</v>
+        <v>46209</v>
       </c>
       <c r="B1141">
-        <v>3080</v>
+        <v>3105</v>
       </c>
       <c r="C1141">
-        <v>13298.5</v>
+        <v>13310</v>
       </c>
       <c r="D1141">
-        <v>1851</v>
+        <v>1852.5</v>
       </c>
       <c r="E1141">
-        <v>16115</v>
+        <v>16065</v>
       </c>
       <c r="F1141">
-        <v>3546</v>
+        <v>3599</v>
       </c>
       <c r="G1141">
-        <v>52000</v>
+        <v>52525</v>
       </c>
     </row>
     <row r="1142" spans="1:7">
       <c r="A1142" s="2">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="B1142">
-        <v>3105</v>
+        <v>3119</v>
       </c>
       <c r="C1142">
-        <v>13310</v>
+        <v>13309</v>
       </c>
       <c r="D1142">
-        <v>1852.5</v>
+        <v>1849</v>
       </c>
       <c r="E1142">
-        <v>16065</v>
+        <v>16160</v>
       </c>
       <c r="F1142">
-        <v>3599</v>
+        <v>3560</v>
       </c>
       <c r="G1142">
-        <v>52525</v>
+        <v>52900</v>
       </c>
     </row>
     <row r="1143" spans="1:7">
       <c r="A1143" s="2">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="B1143">
-        <v>3119</v>
+        <v>3141</v>
       </c>
       <c r="C1143">
-        <v>13309</v>
+        <v>13090</v>
       </c>
       <c r="D1143">
-        <v>1849</v>
+        <v>1851</v>
       </c>
       <c r="E1143">
         <v>16160</v>
       </c>
       <c r="F1143">
-        <v>3560</v>
+        <v>3529</v>
       </c>
       <c r="G1143">
-        <v>52900</v>
+        <v>52350</v>
       </c>
     </row>
     <row r="1144" spans="1:7">
       <c r="A1144" s="2">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B1144">
-        <v>3141</v>
+        <v>3164</v>
       </c>
       <c r="C1144">
-        <v>13090</v>
+        <v>13356.5</v>
       </c>
       <c r="D1144">
-        <v>1851</v>
+        <v>1850</v>
       </c>
       <c r="E1144">
-        <v>16160</v>
+        <v>16355</v>
       </c>
       <c r="F1144">
-        <v>3529</v>
+        <v>3622</v>
       </c>
       <c r="G1144">
-        <v>52350</v>
+        <v>53450</v>
       </c>
     </row>
     <row r="1145" spans="1:7">
       <c r="A1145" s="2">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="B1145">
-        <v>3164</v>
+        <v>3156</v>
       </c>
       <c r="C1145">
-        <v>13356.5</v>
+        <v>13408.5</v>
       </c>
       <c r="D1145">
-        <v>1850</v>
+        <v>1851</v>
       </c>
       <c r="E1145">
-        <v>16355</v>
+        <v>16410</v>
       </c>
       <c r="F1145">
-        <v>3622</v>
+        <v>3602</v>
       </c>
       <c r="G1145">
-        <v>53450</v>
+        <v>52575</v>
       </c>
     </row>
     <row r="1146" spans="1:7">
       <c r="A1146" s="2">
-        <v>46213</v>
+        <v>46216</v>
       </c>
       <c r="B1146">
-        <v>3156</v>
+        <v>3138.5</v>
       </c>
       <c r="C1146">
-        <v>13408.5</v>
+        <v>13460.5</v>
       </c>
       <c r="D1146">
-        <v>1851</v>
+        <v>1832</v>
       </c>
       <c r="E1146">
-        <v>16410</v>
+        <v>16405</v>
       </c>
       <c r="F1146">
-        <v>3602</v>
+        <v>3571</v>
       </c>
       <c r="G1146">
-        <v>52575</v>
+        <v>52705</v>
       </c>
     </row>
     <row r="1147" spans="1:7">
       <c r="A1147" s="2">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="B1147">
-        <v>3138.5</v>
+        <v>3171</v>
       </c>
       <c r="C1147">
-        <v>13460.5</v>
+        <v>13541</v>
       </c>
       <c r="D1147">
-        <v>1832</v>
+        <v>1803</v>
       </c>
       <c r="E1147">
-        <v>16405</v>
+        <v>16590</v>
       </c>
       <c r="F1147">
-        <v>3571</v>
+        <v>3589.5</v>
       </c>
       <c r="G1147">
-        <v>52705</v>
+        <v>53900</v>
       </c>
     </row>
     <row r="1148" spans="1:7">
       <c r="A1148" s="2">
-        <v>46217</v>
+        <v>46218</v>
       </c>
       <c r="B1148">
-        <v>3171</v>
+        <v>3153.5</v>
       </c>
       <c r="C1148">
-        <v>13541</v>
+        <v>13537</v>
       </c>
       <c r="D1148">
-        <v>1803</v>
+        <v>1797</v>
       </c>
       <c r="E1148">
-        <v>16590</v>
+        <v>16505</v>
       </c>
       <c r="F1148">
-        <v>3589.5</v>
+        <v>3553.5</v>
       </c>
       <c r="G1148">
-        <v>53900</v>
+        <v>52705</v>
       </c>
     </row>
     <row r="1149" spans="1:7">
       <c r="A1149" s="2">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="B1149">
-        <v>3153.5</v>
+        <v>3170</v>
       </c>
       <c r="C1149">
-        <v>13537</v>
+        <v>13565</v>
       </c>
       <c r="D1149">
-        <v>1797</v>
+        <v>1827.5</v>
       </c>
       <c r="E1149">
-        <v>16505</v>
+        <v>17150</v>
       </c>
       <c r="F1149">
-        <v>3553.5</v>
+        <v>3591</v>
       </c>
       <c r="G1149">
-        <v>52705</v>
+        <v>52860</v>
       </c>
     </row>
     <row r="1150" spans="1:7">
       <c r="A1150" s="2">
-        <v>46219</v>
+        <v>46220</v>
       </c>
       <c r="B1150">
-        <v>3170</v>
+        <v>3154</v>
       </c>
       <c r="C1150">
-        <v>13565</v>
+        <v>13373.5</v>
       </c>
       <c r="D1150">
-        <v>1827.5</v>
+        <v>1821</v>
       </c>
       <c r="E1150">
-        <v>17150</v>
+        <v>16725</v>
       </c>
       <c r="F1150">
-        <v>3591</v>
+        <v>3549</v>
       </c>
       <c r="G1150">
-        <v>52860</v>
+        <v>52045</v>
       </c>
     </row>
     <row r="1151" spans="1:7">
       <c r="A1151" s="2">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="B1151">
-        <v>3154</v>
+        <v>3156</v>
       </c>
       <c r="C1151">
-        <v>13373.5</v>
+        <v>13629</v>
       </c>
       <c r="D1151">
-        <v>1821</v>
+        <v>1830</v>
       </c>
       <c r="E1151">
-        <v>16725</v>
+        <v>16850</v>
       </c>
       <c r="F1151">
-        <v>3549</v>
+        <v>3575</v>
       </c>
       <c r="G1151">
-        <v>52045</v>
+        <v>53300</v>
       </c>
     </row>
     <row r="1152" spans="1:7">
       <c r="A1152" s="2">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="B1152">
-        <v>3156</v>
+        <v>3183.5</v>
       </c>
       <c r="C1152">
-        <v>13629</v>
+        <v>13856</v>
       </c>
       <c r="D1152">
-        <v>1830</v>
+        <v>1842</v>
       </c>
       <c r="E1152">
-        <v>16850</v>
+        <v>16970</v>
       </c>
       <c r="F1152">
-        <v>3575</v>
+        <v>3591</v>
       </c>
       <c r="G1152">
-        <v>53300</v>
+        <v>54100</v>
       </c>
     </row>
     <row r="1153" spans="1:7">
       <c r="A1153" s="2">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="B1153">
-        <v>3183.5</v>
+        <v>3205</v>
       </c>
       <c r="C1153">
-        <v>13856</v>
+        <v>13895</v>
       </c>
       <c r="D1153">
-        <v>1842</v>
+        <v>1841.5</v>
       </c>
       <c r="E1153">
-        <v>16970</v>
+        <v>16940</v>
       </c>
       <c r="F1153">
-        <v>3591</v>
+        <v>3614</v>
       </c>
       <c r="G1153">
-        <v>54100</v>
+        <v>53900</v>
       </c>
     </row>
     <row r="1154" spans="1:7">
       <c r="A1154" s="2">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="B1154">
-        <v>3205</v>
+        <v>3194</v>
       </c>
       <c r="C1154">
-        <v>13895</v>
+        <v>13745</v>
       </c>
       <c r="D1154">
-        <v>1841.5</v>
+        <v>1875</v>
       </c>
       <c r="E1154">
-        <v>16940</v>
+        <v>17200</v>
       </c>
       <c r="F1154">
-        <v>3614</v>
+        <v>3653</v>
       </c>
       <c r="G1154">
-        <v>53900</v>
+        <v>53800</v>
       </c>
     </row>
     <row r="1155" spans="1:7">
       <c r="A1155" s="2">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="B1155">
-        <v>3194</v>
+        <v>3175</v>
       </c>
       <c r="C1155">
-        <v>13745</v>
+        <v>13617</v>
       </c>
       <c r="D1155">
-        <v>1875</v>
+        <v>1865.5</v>
       </c>
       <c r="E1155">
-        <v>17200</v>
+        <v>17205</v>
       </c>
       <c r="F1155">
-        <v>3653</v>
+        <v>3633</v>
       </c>
       <c r="G1155">
-        <v>53800</v>
+        <v>53250</v>
       </c>
     </row>
     <row r="1156" spans="1:7">
       <c r="A1156" s="2">
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="B1156">
-        <v>3175</v>
+        <v>3192</v>
       </c>
       <c r="C1156">
-        <v>13617</v>
+        <v>13810</v>
       </c>
       <c r="D1156">
-        <v>1865.5</v>
+        <v>1859</v>
       </c>
       <c r="E1156">
-        <v>17205</v>
+        <v>17165</v>
       </c>
       <c r="F1156">
-        <v>3633</v>
+        <v>3685.5</v>
       </c>
       <c r="G1156">
-        <v>53250</v>
+        <v>54250</v>
       </c>
     </row>
     <row r="1157" spans="1:7">
       <c r="A1157" s="2">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B1157">
-        <v>3192</v>
+        <v>3159.5</v>
       </c>
       <c r="C1157">
-        <v>13810</v>
+        <v>13643.5</v>
       </c>
       <c r="D1157">
-        <v>1859</v>
+        <v>1856</v>
       </c>
       <c r="E1157">
-        <v>17165</v>
+        <v>16860</v>
       </c>
       <c r="F1157">
-        <v>3685.5</v>
+        <v>3631.5</v>
       </c>
       <c r="G1157">
-        <v>54250</v>
+        <v>53600</v>
       </c>
     </row>
     <row r="1158" spans="1:7">
       <c r="A1158" s="2">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B1158">
-        <v>3159.5</v>
+        <v>3207</v>
       </c>
       <c r="C1158">
-        <v>13643.5</v>
+        <v>13633</v>
       </c>
       <c r="D1158">
-        <v>1856</v>
+        <v>1877</v>
       </c>
       <c r="E1158">
-        <v>16860</v>
+        <v>17000</v>
       </c>
       <c r="F1158">
-        <v>3631.5</v>
+        <v>3639</v>
       </c>
       <c r="G1158">
-        <v>53600</v>
+        <v>53990</v>
       </c>
     </row>
     <row r="1159" spans="1:7">
       <c r="A1159" s="2">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B1159">
-        <v>3207</v>
+        <v>3231</v>
       </c>
       <c r="C1159">
-        <v>13633</v>
+        <v>13795</v>
       </c>
       <c r="D1159">
-        <v>1877</v>
+        <v>1863</v>
       </c>
       <c r="E1159">
-        <v>17000</v>
+        <v>16945</v>
       </c>
       <c r="F1159">
-        <v>3639</v>
+        <v>3662</v>
       </c>
       <c r="G1159">
-        <v>53990</v>
+        <v>54125</v>
       </c>
     </row>
     <row r="1160" spans="1:7">
       <c r="A1160" s="2">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="B1160">
-        <v>3231</v>
+        <v>3196</v>
       </c>
       <c r="C1160">
-        <v>13795</v>
+        <v>13834</v>
       </c>
       <c r="D1160">
-        <v>1863</v>
+        <v>1851.5</v>
       </c>
       <c r="E1160">
-        <v>16945</v>
+        <v>17100</v>
       </c>
       <c r="F1160">
-        <v>3662</v>
+        <v>3710.5</v>
       </c>
       <c r="G1160">
-        <v>54125</v>
+        <v>54660</v>
       </c>
     </row>
     <row r="1161" spans="1:7">
       <c r="A1161" s="2">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="B1161">
-        <v>3196</v>
+        <v>3260</v>
       </c>
       <c r="C1161">
-        <v>13834</v>
+        <v>13945</v>
       </c>
       <c r="D1161">
-        <v>1851.5</v>
+        <v>1828</v>
       </c>
       <c r="E1161">
-        <v>17100</v>
+        <v>16785</v>
       </c>
       <c r="F1161">
-        <v>3710.5</v>
+        <v>3751</v>
       </c>
       <c r="G1161">
-        <v>54660</v>
+        <v>55200</v>
       </c>
     </row>
     <row r="1162" spans="1:7">
       <c r="A1162" s="2">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B1162">
-        <v>3260</v>
+        <v>3271</v>
       </c>
       <c r="C1162">
-        <v>13945</v>
+        <v>14195</v>
       </c>
       <c r="D1162">
-        <v>1828</v>
+        <v>1847</v>
       </c>
       <c r="E1162">
-        <v>16785</v>
+        <v>17125</v>
       </c>
       <c r="F1162">
-        <v>3751</v>
+        <v>3730</v>
       </c>
       <c r="G1162">
-        <v>55200</v>
+        <v>55700</v>
       </c>
     </row>
     <row r="1163" spans="1:7">
       <c r="A1163" s="2">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="B1163">
-        <v>3271</v>
+        <v>3229</v>
       </c>
       <c r="C1163">
-        <v>14195</v>
+        <v>14167.5</v>
       </c>
       <c r="D1163">
-        <v>1847</v>
+        <v>1845</v>
       </c>
       <c r="E1163">
-        <v>17125</v>
+        <v>16915</v>
       </c>
       <c r="F1163">
-        <v>3730</v>
+        <v>3737</v>
       </c>
       <c r="G1163">
-        <v>55700</v>
+        <v>56225</v>
       </c>
     </row>
     <row r="1164" spans="1:7">
       <c r="A1164" s="2">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="B1164">
-        <v>3229</v>
+        <v>3261</v>
       </c>
       <c r="C1164">
-        <v>14167.5</v>
+        <v>14455</v>
       </c>
       <c r="D1164">
-        <v>1845</v>
+        <v>1851</v>
       </c>
       <c r="E1164">
-        <v>16915</v>
+        <v>16595</v>
       </c>
       <c r="F1164">
-        <v>3737</v>
+        <v>3857</v>
       </c>
       <c r="G1164">
-        <v>56225</v>
+        <v>56500</v>
       </c>
     </row>
     <row r="1165" spans="1:7">
       <c r="A1165" s="2">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="B1165">
-        <v>3261</v>
+        <v>3279.5</v>
       </c>
       <c r="C1165">
-        <v>14455</v>
+        <v>14240</v>
       </c>
       <c r="D1165">
-        <v>1851</v>
+        <v>1840.5</v>
       </c>
       <c r="E1165">
-        <v>16595</v>
+        <v>16745</v>
       </c>
       <c r="F1165">
-        <v>3857</v>
+        <v>3785</v>
       </c>
       <c r="G1165">
-        <v>56500</v>
+        <v>56100</v>
       </c>
     </row>
     <row r="1166" spans="1:7">
       <c r="A1166" s="2">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="B1166">
-        <v>3279.5</v>
+        <v>3327.5</v>
       </c>
       <c r="C1166">
-        <v>14240</v>
+        <v>14290</v>
       </c>
       <c r="D1166">
-        <v>1840.5</v>
+        <v>1858</v>
       </c>
       <c r="E1166">
-        <v>16745</v>
+        <v>16775</v>
       </c>
       <c r="F1166">
-        <v>3785</v>
+        <v>3786</v>
       </c>
       <c r="G1166">
-        <v>56100</v>
+        <v>55900</v>
       </c>
     </row>
     <row r="1167" spans="1:7">
       <c r="A1167" s="2">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="B1167">
-        <v>3327.5</v>
+        <v>3373</v>
       </c>
       <c r="C1167">
-        <v>14290</v>
+        <v>14424.5</v>
       </c>
       <c r="D1167">
-        <v>1858</v>
+        <v>1878</v>
       </c>
       <c r="E1167">
-        <v>16775</v>
+        <v>16640</v>
       </c>
       <c r="F1167">
-        <v>3786</v>
+        <v>3822</v>
       </c>
       <c r="G1167">
-        <v>55900</v>
+        <v>55305</v>
       </c>
     </row>
     <row r="1168" spans="1:7">
       <c r="A1168" s="2">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="B1168">
-        <v>3373</v>
+        <v>3307.5</v>
       </c>
       <c r="C1168">
-        <v>14424.5</v>
+        <v>14376</v>
       </c>
       <c r="D1168">
-        <v>1878</v>
+        <v>1880</v>
       </c>
       <c r="E1168">
-        <v>16640</v>
+        <v>16725</v>
       </c>
       <c r="F1168">
-        <v>3822</v>
+        <v>3852</v>
       </c>
       <c r="G1168">
-        <v>55305</v>
+        <v>56050</v>
       </c>
     </row>
     <row r="1169" spans="1:7">
       <c r="A1169" s="2">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="B1169">
-        <v>3307.5</v>
+        <v>3279</v>
       </c>
       <c r="C1169">
-        <v>14376</v>
+        <v>14285</v>
       </c>
       <c r="D1169">
-        <v>1880</v>
+        <v>1856</v>
       </c>
       <c r="E1169">
-        <v>16725</v>
+        <v>16690</v>
       </c>
       <c r="F1169">
-        <v>3852</v>
+        <v>3806</v>
       </c>
       <c r="G1169">
-        <v>56050</v>
+        <v>56150</v>
       </c>
     </row>
     <row r="1170" spans="1:7">
       <c r="A1170" s="2">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="B1170">
-        <v>3279</v>
+        <v>3248</v>
       </c>
       <c r="C1170">
-        <v>14285</v>
+        <v>14545</v>
       </c>
       <c r="D1170">
-        <v>1856</v>
+        <v>1846</v>
       </c>
       <c r="E1170">
-        <v>16690</v>
+        <v>16575</v>
       </c>
       <c r="F1170">
-        <v>3806</v>
+        <v>3875</v>
       </c>
       <c r="G1170">
-        <v>56150</v>
+        <v>56075</v>
       </c>
     </row>
     <row r="1171" spans="1:7">
       <c r="A1171" s="2">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="B1171">
-        <v>3248</v>
+        <v>3272</v>
       </c>
       <c r="C1171">
-        <v>14545</v>
+        <v>14850</v>
       </c>
       <c r="D1171">
-        <v>1846</v>
+        <v>1851.5</v>
       </c>
       <c r="E1171">
-        <v>16575</v>
+        <v>16670</v>
       </c>
       <c r="F1171">
-        <v>3875</v>
+        <v>3855</v>
       </c>
       <c r="G1171">
-        <v>56075</v>
+        <v>56225</v>
       </c>
     </row>
     <row r="1172" spans="1:7">
       <c r="A1172" s="2">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="B1172">
-        <v>3272</v>
+        <v>3219</v>
       </c>
       <c r="C1172">
-        <v>14850</v>
+        <v>14335</v>
       </c>
       <c r="D1172">
-        <v>1851.5</v>
+        <v>1840.5</v>
       </c>
       <c r="E1172">
-        <v>16670</v>
+        <v>16740</v>
       </c>
       <c r="F1172">
-        <v>3855</v>
+        <v>3795</v>
       </c>
       <c r="G1172">
-        <v>56225</v>
+        <v>55550</v>
       </c>
     </row>
     <row r="1173" spans="1:7">
       <c r="A1173" s="2">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="B1173">
-        <v>3219</v>
+        <v>3191.5</v>
       </c>
       <c r="C1173">
-        <v>14335</v>
+        <v>14180</v>
       </c>
       <c r="D1173">
-        <v>1840.5</v>
+        <v>1827</v>
       </c>
       <c r="E1173">
-        <v>16740</v>
+        <v>16690</v>
       </c>
       <c r="F1173">
-        <v>3795</v>
+        <v>3750</v>
       </c>
       <c r="G1173">
-        <v>55550</v>
+        <v>54375</v>
       </c>
     </row>
     <row r="1174" spans="1:7">
       <c r="A1174" s="2">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="B1174">
-        <v>3191.5</v>
+        <v>3182</v>
       </c>
       <c r="C1174">
-        <v>14180</v>
+        <v>14170</v>
       </c>
       <c r="D1174">
-        <v>1827</v>
+        <v>1848</v>
       </c>
       <c r="E1174">
-        <v>16690</v>
+        <v>16660</v>
       </c>
       <c r="F1174">
-        <v>3750</v>
+        <v>3865.5</v>
       </c>
       <c r="G1174">
-        <v>54375</v>
+        <v>54850</v>
       </c>
     </row>
     <row r="1175" spans="1:7">
       <c r="A1175" s="2">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="B1175">
-        <v>3182</v>
+        <v>3227</v>
       </c>
       <c r="C1175">
-        <v>14170</v>
+        <v>14291</v>
       </c>
       <c r="D1175">
-        <v>1848</v>
+        <v>1857</v>
       </c>
       <c r="E1175">
-        <v>16660</v>
+        <v>16860</v>
       </c>
       <c r="F1175">
-        <v>3865.5</v>
+        <v>3980</v>
       </c>
       <c r="G1175">
-        <v>54850</v>
+        <v>55900</v>
       </c>
     </row>
     <row r="1176" spans="1:7">
       <c r="A1176" s="2">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="B1176">
-        <v>3227</v>
+        <v>3215.5</v>
       </c>
       <c r="C1176">
-        <v>14291</v>
+        <v>14344</v>
       </c>
       <c r="D1176">
-        <v>1857</v>
+        <v>1862.5</v>
       </c>
       <c r="E1176">
-        <v>16860</v>
+        <v>16940</v>
       </c>
       <c r="F1176">
-        <v>3980</v>
+        <v>3985</v>
       </c>
       <c r="G1176">
         <v>55900</v>
@@ -27449,622 +27449,599 @@
     </row>
     <row r="1177" spans="1:7">
       <c r="A1177" s="2">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="B1177">
-        <v>3215.5</v>
+        <v>3188</v>
       </c>
       <c r="C1177">
-        <v>14344</v>
+        <v>14425</v>
       </c>
       <c r="D1177">
-        <v>1862.5</v>
+        <v>1867</v>
       </c>
       <c r="E1177">
-        <v>16940</v>
+        <v>16780</v>
       </c>
       <c r="F1177">
-        <v>3985</v>
+        <v>3987</v>
       </c>
       <c r="G1177">
-        <v>55900</v>
+        <v>55700</v>
       </c>
     </row>
     <row r="1178" spans="1:7">
       <c r="A1178" s="2">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="B1178">
-        <v>3188</v>
+        <v>3227.5</v>
       </c>
       <c r="C1178">
-        <v>14425</v>
+        <v>14525</v>
       </c>
       <c r="D1178">
-        <v>1867</v>
+        <v>1866</v>
       </c>
       <c r="E1178">
-        <v>16780</v>
+        <v>16895</v>
       </c>
       <c r="F1178">
-        <v>3987</v>
+        <v>4107</v>
       </c>
       <c r="G1178">
-        <v>55700</v>
+        <v>55300</v>
       </c>
     </row>
     <row r="1179" spans="1:7">
       <c r="A1179" s="2">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="B1179">
-        <v>3227.5</v>
+        <v>3212.5</v>
       </c>
       <c r="C1179">
-        <v>14525</v>
+        <v>14490</v>
       </c>
       <c r="D1179">
-        <v>1866</v>
+        <v>1872</v>
       </c>
       <c r="E1179">
-        <v>16895</v>
+        <v>16660</v>
       </c>
       <c r="F1179">
         <v>4107</v>
       </c>
       <c r="G1179">
-        <v>55300</v>
+        <v>54950</v>
       </c>
     </row>
     <row r="1180" spans="1:7">
       <c r="A1180" s="2">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="B1180">
-        <v>3212.5</v>
+        <v>3222</v>
       </c>
       <c r="C1180">
-        <v>14490</v>
+        <v>14535</v>
       </c>
       <c r="D1180">
-        <v>1872</v>
+        <v>1880</v>
       </c>
       <c r="E1180">
-        <v>16660</v>
+        <v>16850</v>
       </c>
       <c r="F1180">
-        <v>4107</v>
+        <v>4070</v>
       </c>
       <c r="G1180">
-        <v>54950</v>
+        <v>55125</v>
       </c>
     </row>
     <row r="1181" spans="1:7">
       <c r="A1181" s="2">
-        <v>46262</v>
+        <v>46266</v>
       </c>
       <c r="B1181">
-        <v>3222</v>
+        <v>3261</v>
       </c>
       <c r="C1181">
-        <v>14535</v>
+        <v>14395.5</v>
       </c>
       <c r="D1181">
-        <v>1880</v>
+        <v>1874</v>
       </c>
       <c r="E1181">
-        <v>16850</v>
+        <v>16350</v>
       </c>
       <c r="F1181">
-        <v>4070</v>
+        <v>4115</v>
       </c>
       <c r="G1181">
-        <v>55125</v>
+        <v>54725</v>
       </c>
     </row>
     <row r="1182" spans="1:7">
       <c r="A1182" s="2">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="B1182">
-        <v>3261</v>
+        <v>3255.5</v>
       </c>
       <c r="C1182">
-        <v>14395.5</v>
+        <v>14355</v>
       </c>
       <c r="D1182">
-        <v>1874</v>
+        <v>1873</v>
       </c>
       <c r="E1182">
-        <v>16350</v>
+        <v>16530</v>
       </c>
       <c r="F1182">
-        <v>4115</v>
+        <v>4000</v>
       </c>
       <c r="G1182">
-        <v>54725</v>
+        <v>53950</v>
       </c>
     </row>
     <row r="1183" spans="1:7">
       <c r="A1183" s="2">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="B1183">
-        <v>3255.5</v>
+        <v>3303</v>
       </c>
       <c r="C1183">
-        <v>14355</v>
+        <v>14359</v>
       </c>
       <c r="D1183">
-        <v>1873</v>
+        <v>1870</v>
       </c>
       <c r="E1183">
-        <v>16530</v>
+        <v>16615</v>
       </c>
       <c r="F1183">
-        <v>4000</v>
+        <v>3995.5</v>
       </c>
       <c r="G1183">
-        <v>53950</v>
+        <v>54450</v>
       </c>
     </row>
     <row r="1184" spans="1:7">
       <c r="A1184" s="2">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="B1184">
-        <v>3303</v>
+        <v>3292.5</v>
       </c>
       <c r="C1184">
-        <v>14359</v>
+        <v>14371</v>
       </c>
       <c r="D1184">
-        <v>1870</v>
+        <v>1871</v>
       </c>
       <c r="E1184">
-        <v>16615</v>
+        <v>16690</v>
       </c>
       <c r="F1184">
-        <v>3995.5</v>
+        <v>4087</v>
       </c>
       <c r="G1184">
-        <v>54450</v>
+        <v>54525</v>
       </c>
     </row>
     <row r="1185" spans="1:7">
       <c r="A1185" s="2">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B1185">
-        <v>3292.5</v>
+        <v>3310</v>
       </c>
       <c r="C1185">
-        <v>14371</v>
+        <v>14540</v>
       </c>
       <c r="D1185">
-        <v>1871</v>
+        <v>1875</v>
       </c>
       <c r="E1185">
-        <v>16690</v>
+        <v>16600</v>
       </c>
       <c r="F1185">
-        <v>4087</v>
+        <v>4157</v>
       </c>
       <c r="G1185">
-        <v>54525</v>
+        <v>55100</v>
       </c>
     </row>
     <row r="1186" spans="1:7">
       <c r="A1186" s="2">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B1186">
-        <v>3310</v>
+        <v>3325</v>
       </c>
       <c r="C1186">
-        <v>14540</v>
+        <v>14737</v>
       </c>
       <c r="D1186">
-        <v>1875</v>
+        <v>1859</v>
       </c>
       <c r="E1186">
-        <v>16600</v>
+        <v>16675</v>
       </c>
       <c r="F1186">
-        <v>4157</v>
+        <v>4110</v>
       </c>
       <c r="G1186">
-        <v>55100</v>
+        <v>54900</v>
       </c>
     </row>
     <row r="1187" spans="1:7">
       <c r="A1187" s="2">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B1187">
-        <v>3325</v>
+        <v>3352</v>
       </c>
       <c r="C1187">
-        <v>14737</v>
+        <v>14672</v>
       </c>
       <c r="D1187">
-        <v>1859</v>
+        <v>1871</v>
       </c>
       <c r="E1187">
         <v>16675</v>
       </c>
       <c r="F1187">
-        <v>4110</v>
+        <v>4186</v>
       </c>
       <c r="G1187">
-        <v>54900</v>
+        <v>55000</v>
       </c>
     </row>
     <row r="1188" spans="1:7">
       <c r="A1188" s="2">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="B1188">
-        <v>3352</v>
+        <v>3343</v>
       </c>
       <c r="C1188">
-        <v>14672</v>
+        <v>14390</v>
       </c>
       <c r="D1188">
-        <v>1871</v>
+        <v>1870.5</v>
       </c>
       <c r="E1188">
-        <v>16675</v>
+        <v>16630</v>
       </c>
       <c r="F1188">
-        <v>4186</v>
+        <v>4105</v>
       </c>
       <c r="G1188">
-        <v>55000</v>
+        <v>54750</v>
       </c>
     </row>
     <row r="1189" spans="1:7">
       <c r="A1189" s="2">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B1189">
-        <v>3343</v>
+        <v>3274</v>
       </c>
       <c r="C1189">
-        <v>14390</v>
+        <v>14238.5</v>
       </c>
       <c r="D1189">
-        <v>1870.5</v>
+        <v>1854</v>
       </c>
       <c r="E1189">
-        <v>16630</v>
+        <v>16270</v>
       </c>
       <c r="F1189">
-        <v>4105</v>
+        <v>4015</v>
       </c>
       <c r="G1189">
-        <v>54750</v>
+        <v>53755</v>
       </c>
     </row>
     <row r="1190" spans="1:7">
       <c r="A1190" s="2">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="B1190">
-        <v>3274</v>
+        <v>3311</v>
       </c>
       <c r="C1190">
-        <v>14238.5</v>
+        <v>14044</v>
       </c>
       <c r="D1190">
-        <v>1854</v>
+        <v>1834</v>
       </c>
       <c r="E1190">
-        <v>16270</v>
+        <v>16205</v>
       </c>
       <c r="F1190">
-        <v>4015</v>
+        <v>3951</v>
       </c>
       <c r="G1190">
-        <v>53755</v>
+        <v>52200</v>
       </c>
     </row>
     <row r="1191" spans="1:7">
       <c r="A1191" s="2">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="B1191">
-        <v>3311</v>
+        <v>3260</v>
       </c>
       <c r="C1191">
-        <v>14044</v>
+        <v>14045</v>
       </c>
       <c r="D1191">
-        <v>1834</v>
+        <v>1829</v>
       </c>
       <c r="E1191">
-        <v>16205</v>
+        <v>16135</v>
       </c>
       <c r="F1191">
-        <v>3951</v>
+        <v>3922</v>
       </c>
       <c r="G1191">
-        <v>52200</v>
+        <v>51800</v>
       </c>
     </row>
     <row r="1192" spans="1:7">
       <c r="A1192" s="2">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B1192">
-        <v>3260</v>
+        <v>3310</v>
       </c>
       <c r="C1192">
-        <v>14045</v>
+        <v>14227</v>
       </c>
       <c r="D1192">
-        <v>1829</v>
+        <v>1848</v>
       </c>
       <c r="E1192">
-        <v>16135</v>
+        <v>16090</v>
       </c>
       <c r="F1192">
-        <v>3922</v>
+        <v>3937</v>
       </c>
       <c r="G1192">
-        <v>51800</v>
+        <v>52310</v>
       </c>
     </row>
     <row r="1193" spans="1:7">
       <c r="A1193" s="2">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B1193">
-        <v>3310</v>
+        <v>3303.5</v>
       </c>
       <c r="C1193">
-        <v>14227</v>
+        <v>14400.5</v>
       </c>
       <c r="D1193">
-        <v>1848</v>
+        <v>1862</v>
       </c>
       <c r="E1193">
-        <v>16090</v>
+        <v>16170</v>
       </c>
       <c r="F1193">
-        <v>3937</v>
+        <v>3941</v>
       </c>
       <c r="G1193">
-        <v>52310</v>
+        <v>53000</v>
       </c>
     </row>
     <row r="1194" spans="1:7">
       <c r="A1194" s="2">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B1194">
-        <v>3303.5</v>
+        <v>3285</v>
       </c>
       <c r="C1194">
-        <v>14400.5</v>
+        <v>14529</v>
       </c>
       <c r="D1194">
-        <v>1862</v>
+        <v>1868</v>
       </c>
       <c r="E1194">
-        <v>16170</v>
+        <v>16055</v>
       </c>
       <c r="F1194">
-        <v>3941</v>
+        <v>4010</v>
       </c>
       <c r="G1194">
-        <v>53000</v>
+        <v>53600</v>
       </c>
     </row>
     <row r="1195" spans="1:7">
       <c r="A1195" s="2">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="B1195">
-        <v>3285</v>
+        <v>3262.5</v>
       </c>
       <c r="C1195">
-        <v>14529</v>
+        <v>14788</v>
       </c>
       <c r="D1195">
-        <v>1868</v>
+        <v>1890</v>
       </c>
       <c r="E1195">
-        <v>16055</v>
+        <v>16125</v>
       </c>
       <c r="F1195">
-        <v>4010</v>
+        <v>4018</v>
       </c>
       <c r="G1195">
-        <v>53600</v>
+        <v>53785</v>
       </c>
     </row>
     <row r="1196" spans="1:7">
       <c r="A1196" s="2">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="B1196">
-        <v>3262.5</v>
+        <v>3242</v>
       </c>
       <c r="C1196">
-        <v>14788</v>
+        <v>14797</v>
       </c>
       <c r="D1196">
-        <v>1890</v>
+        <v>1909</v>
       </c>
       <c r="E1196">
-        <v>16125</v>
+        <v>16410</v>
       </c>
       <c r="F1196">
-        <v>4018</v>
+        <v>4006</v>
       </c>
       <c r="G1196">
-        <v>53785</v>
+        <v>53745</v>
       </c>
     </row>
     <row r="1197" spans="1:7">
       <c r="A1197" s="2">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B1197">
-        <v>3242</v>
+        <v>3240</v>
       </c>
       <c r="C1197">
-        <v>14797</v>
+        <v>14735</v>
       </c>
       <c r="D1197">
-        <v>1909</v>
+        <v>1885.5</v>
       </c>
       <c r="E1197">
-        <v>16410</v>
+        <v>16430</v>
       </c>
       <c r="F1197">
-        <v>4006</v>
+        <v>3949</v>
       </c>
       <c r="G1197">
-        <v>53745</v>
+        <v>54050</v>
       </c>
     </row>
     <row r="1198" spans="1:7">
       <c r="A1198" s="2">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B1198">
-        <v>3240</v>
+        <v>3228</v>
       </c>
       <c r="C1198">
-        <v>14735</v>
+        <v>14765</v>
       </c>
       <c r="D1198">
-        <v>1885.5</v>
+        <v>1900</v>
       </c>
       <c r="E1198">
-        <v>16430</v>
+        <v>16320</v>
       </c>
       <c r="F1198">
-        <v>3949</v>
+        <v>3981</v>
       </c>
       <c r="G1198">
-        <v>54050</v>
+        <v>53875</v>
       </c>
     </row>
     <row r="1199" spans="1:7">
       <c r="A1199" s="2">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B1199">
-        <v>3228</v>
+        <v>3254</v>
       </c>
       <c r="C1199">
-        <v>14765</v>
+        <v>14740</v>
       </c>
       <c r="D1199">
-        <v>1900</v>
+        <v>1902.5</v>
       </c>
       <c r="E1199">
-        <v>16320</v>
+        <v>16050</v>
       </c>
       <c r="F1199">
-        <v>3981</v>
+        <v>4060</v>
       </c>
       <c r="G1199">
-        <v>53875</v>
+        <v>54025</v>
       </c>
     </row>
     <row r="1200" spans="1:7">
       <c r="A1200" s="2">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="B1200">
-        <v>3254</v>
+        <v>3248.5</v>
       </c>
       <c r="C1200">
-        <v>14740</v>
+        <v>14544.5</v>
       </c>
       <c r="D1200">
-        <v>1902.5</v>
+        <v>1886</v>
       </c>
       <c r="E1200">
         <v>16050</v>
       </c>
       <c r="F1200">
-        <v>4060</v>
+        <v>3957</v>
       </c>
       <c r="G1200">
-        <v>54025</v>
+        <v>53750</v>
       </c>
     </row>
     <row r="1201" spans="1:7">
       <c r="A1201" s="2">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="B1201">
-        <v>3248.5</v>
+        <v>3225.5</v>
       </c>
       <c r="C1201">
-        <v>14544.5</v>
+        <v>14474.5</v>
       </c>
       <c r="D1201">
-        <v>1886</v>
+        <v>1876</v>
       </c>
       <c r="E1201">
-        <v>16050</v>
+        <v>15860</v>
       </c>
       <c r="F1201">
-        <v>3957</v>
+        <v>3977</v>
       </c>
       <c r="G1201">
-        <v>53750</v>
+        <v>53950</v>
       </c>
     </row>
     <row r="1202" spans="1:7">
       <c r="A1202" s="2">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B1202">
-        <v>3225.5</v>
+        <v>3204</v>
       </c>
       <c r="C1202">
-        <v>14474.5</v>
+        <v>14487</v>
       </c>
       <c r="D1202">
-        <v>1876</v>
+        <v>1856</v>
       </c>
       <c r="E1202">
         <v>15860</v>
       </c>
       <c r="F1202">
-        <v>3977</v>
+        <v>3954</v>
       </c>
       <c r="G1202">
-        <v>53950</v>
-      </c>
-    </row>
-    <row r="1203" spans="1:7">
-      <c r="A1203" s="2">
-        <v>46295</v>
-      </c>
-      <c r="B1203">
-        <v>3204</v>
-      </c>
-      <c r="C1203">
-        <v>14487</v>
-      </c>
-      <c r="D1203">
-        <v>1856</v>
-      </c>
-      <c r="E1203">
-        <v>15860</v>
-      </c>
-      <c r="F1203">
-        <v>3954</v>
-      </c>
-      <c r="G1203">
         <v>54075</v>
       </c>
     </row>

</xml_diff>